<commit_message>
Fix: Añadido packages.txt para instalacion de LibreOffice y exportacion directa a PDF
</commit_message>
<xml_diff>
--- a/PLANTILLA_GR.xlsx
+++ b/PLANTILLA_GR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ct75272700\Desktop\THL\TEMPORALES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TH HABIL\2026\008 AUTOMATIZACION\PDF TO FIRMAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2F42830-3136-45E7-AAB8-A28D4A4DB5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBF2E3C-C161-42D6-ADE5-A5070935351C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1560" windowWidth="38400" windowHeight="19470" tabRatio="830" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="830" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="super" sheetId="2" state="hidden" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="38">
   <si>
     <t>Referencia:</t>
   </si>
@@ -235,18 +235,6 @@
 PLANTA Y PERFIL</t>
   </si>
   <si>
-    <t>ALCANTARILLA 87+412.236 
-DETALLE DE CABEZAL</t>
-  </si>
-  <si>
-    <t>ALCANTARILLA 87+412.236 
-SECCIÓN TIPO Y DETALLES</t>
-  </si>
-  <si>
-    <t>ALCANTARILLA 87+412.236 
-ACERO DE REFUERZO</t>
-  </si>
-  <si>
     <t>TOPOGRAFÍA OSP</t>
   </si>
   <si>
@@ -270,58 +258,6 @@
   </si>
   <si>
     <t>ASSA-ALC055-05-10-001-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-002-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-003-R4</t>
-  </si>
-  <si>
-    <t>ALCANTARILLA 87+412.236 
-DETALLE DE EMPALME</t>
-  </si>
-  <si>
-    <t>ASSA-ALC055-05-10-004-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-005-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-006-R4</t>
-  </si>
-  <si>
-    <t>ASSA-ALC055-05-10-007-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-008-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-009-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-010-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-011-R4</t>
-  </si>
-  <si>
-    <t>ALCANTARILLA 87+412.236 
-DETALLE DE EMPALME DE ACEROS</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-012-R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALCANTARILLA 87+412.236 
-DETALLE: ESTRUCTURA DE DESCARGA </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ASSA-ALC055-05-10-013-R4</t>
-  </si>
-  <si>
-    <t>ALCANTARILLA 87+412.236 
-ACERO DE REFUERZO  ESTRUCTURA DE DESCARGA</t>
   </si>
 </sst>
 </file>
@@ -700,6 +636,249 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -718,9 +897,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -759,9 +935,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -789,243 +962,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2425,9 +2361,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2465,7 +2401,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2571,7 +2507,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2713,7 +2649,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2736,39 +2672,39 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="71" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="80" t="s">
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="81"/>
+      <c r="J2" s="48"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="83"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="50"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="75"/>
-      <c r="H4" s="76"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="43"/>
       <c r="I4" s="5" t="s">
         <v>16</v>
       </c>
@@ -2777,13 +2713,13 @@
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="77"/>
-      <c r="E5" s="78"/>
-      <c r="F5" s="78"/>
-      <c r="G5" s="78"/>
-      <c r="H5" s="79"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="46"/>
       <c r="I5" s="11" t="s">
         <v>30</v>
       </c>
@@ -2792,66 +2728,66 @@
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="84"/>
-      <c r="D6" s="84"/>
-      <c r="E6" s="84"/>
-      <c r="F6" s="84"/>
-      <c r="G6" s="84"/>
-      <c r="H6" s="84"/>
-      <c r="I6" s="84"/>
-      <c r="J6" s="84"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="51"/>
+      <c r="J6" s="51"/>
     </row>
     <row r="7" spans="2:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="85" t="s">
+      <c r="B7" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="85"/>
-      <c r="D7" s="85"/>
-      <c r="E7" s="85"/>
-      <c r="F7" s="85"/>
-      <c r="G7" s="85"/>
-      <c r="H7" s="85"/>
-      <c r="I7" s="85"/>
-      <c r="J7" s="85"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="52"/>
+      <c r="F7" s="52"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="70"/>
-      <c r="D8" s="70"/>
-      <c r="E8" s="70"/>
-      <c r="F8" s="70"/>
-      <c r="G8" s="70"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="70"/>
-      <c r="J8" s="70"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="37"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="37"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="70"/>
-      <c r="C9" s="70"/>
-      <c r="D9" s="70"/>
-      <c r="E9" s="70"/>
-      <c r="F9" s="70"/>
-      <c r="G9" s="70"/>
-      <c r="H9" s="70"/>
-      <c r="I9" s="70"/>
-      <c r="J9" s="70"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
     </row>
     <row r="10" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B10" s="86" t="s">
+      <c r="B10" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="86"/>
-      <c r="D10" s="86" t="s">
+      <c r="C10" s="35"/>
+      <c r="D10" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="86"/>
-      <c r="F10" s="86"/>
-      <c r="G10" s="86"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
       <c r="H10" s="4" t="s">
         <v>1</v>
       </c>
@@ -2863,479 +2799,503 @@
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B27" s="25"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="25"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="25"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B30" s="88" t="s">
+      <c r="B30" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="C30" s="88"/>
-      <c r="D30" s="88"/>
-      <c r="E30" s="88"/>
-      <c r="F30" s="88"/>
-      <c r="G30" s="88"/>
-      <c r="H30" s="88"/>
-      <c r="I30" s="88"/>
-      <c r="J30" s="88"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B31" s="88"/>
-      <c r="C31" s="88"/>
-      <c r="D31" s="88"/>
-      <c r="E31" s="88"/>
-      <c r="F31" s="88"/>
-      <c r="G31" s="88"/>
-      <c r="H31" s="88"/>
-      <c r="I31" s="88"/>
-      <c r="J31" s="88"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B32" s="88"/>
-      <c r="C32" s="88"/>
-      <c r="D32" s="88"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="88"/>
-      <c r="G32" s="88"/>
-      <c r="H32" s="88"/>
-      <c r="I32" s="88"/>
-      <c r="J32" s="88"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B33" s="88"/>
-      <c r="C33" s="88"/>
-      <c r="D33" s="88"/>
-      <c r="E33" s="88"/>
-      <c r="F33" s="88"/>
-      <c r="G33" s="88"/>
-      <c r="H33" s="88"/>
-      <c r="I33" s="88"/>
-      <c r="J33" s="88"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
     </row>
     <row r="34" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="89" t="s">
+      <c r="B34" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C34" s="90"/>
-      <c r="D34" s="90"/>
-      <c r="E34" s="90"/>
-      <c r="F34" s="90"/>
-      <c r="G34" s="90"/>
-      <c r="H34" s="90"/>
-      <c r="I34" s="90"/>
-      <c r="J34" s="91"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="24"/>
     </row>
     <row r="35" spans="2:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="92"/>
-      <c r="C35" s="93"/>
-      <c r="D35" s="93"/>
-      <c r="E35" s="93"/>
-      <c r="F35" s="93"/>
-      <c r="G35" s="93"/>
-      <c r="H35" s="93"/>
-      <c r="I35" s="93"/>
-      <c r="J35" s="94"/>
+      <c r="B35" s="25"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="26"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="26"/>
+      <c r="I35" s="26"/>
+      <c r="J35" s="27"/>
     </row>
     <row r="36" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="95"/>
-      <c r="C36" s="96"/>
-      <c r="D36" s="96"/>
-      <c r="E36" s="96"/>
-      <c r="F36" s="96"/>
-      <c r="G36" s="96"/>
-      <c r="H36" s="96"/>
-      <c r="I36" s="96"/>
-      <c r="J36" s="97"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="29"/>
+      <c r="J36" s="30"/>
     </row>
     <row r="37" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="89" t="s">
+      <c r="B37" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C37" s="90"/>
-      <c r="D37" s="90"/>
-      <c r="E37" s="90"/>
-      <c r="F37" s="90"/>
-      <c r="G37" s="90"/>
-      <c r="H37" s="90"/>
-      <c r="I37" s="90"/>
-      <c r="J37" s="91"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="24"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="92"/>
-      <c r="C38" s="93"/>
-      <c r="D38" s="93"/>
-      <c r="E38" s="93"/>
-      <c r="F38" s="93"/>
-      <c r="G38" s="93"/>
-      <c r="H38" s="93"/>
-      <c r="I38" s="93"/>
-      <c r="J38" s="94"/>
+      <c r="B38" s="25"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26"/>
+      <c r="F38" s="26"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="26"/>
+      <c r="I38" s="26"/>
+      <c r="J38" s="27"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="92"/>
-      <c r="C39" s="93"/>
-      <c r="D39" s="93"/>
-      <c r="E39" s="93"/>
-      <c r="F39" s="93"/>
-      <c r="G39" s="93"/>
-      <c r="H39" s="93"/>
-      <c r="I39" s="93"/>
-      <c r="J39" s="94"/>
+      <c r="B39" s="25"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="26"/>
+      <c r="G39" s="26"/>
+      <c r="H39" s="26"/>
+      <c r="I39" s="26"/>
+      <c r="J39" s="27"/>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B40" s="92"/>
-      <c r="C40" s="93"/>
-      <c r="D40" s="93"/>
-      <c r="E40" s="93"/>
-      <c r="F40" s="93"/>
-      <c r="G40" s="93"/>
-      <c r="H40" s="93"/>
-      <c r="I40" s="93"/>
-      <c r="J40" s="94"/>
+      <c r="B40" s="25"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="26"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="26"/>
+      <c r="J40" s="27"/>
     </row>
     <row r="41" spans="2:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="95"/>
-      <c r="C41" s="96"/>
-      <c r="D41" s="96"/>
-      <c r="E41" s="96"/>
-      <c r="F41" s="96"/>
-      <c r="G41" s="96"/>
-      <c r="H41" s="96"/>
-      <c r="I41" s="96"/>
-      <c r="J41" s="97"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="29"/>
+      <c r="I41" s="29"/>
+      <c r="J41" s="30"/>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B42" s="98" t="s">
+      <c r="B42" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="C42" s="99"/>
-      <c r="D42" s="99"/>
-      <c r="E42" s="99"/>
-      <c r="F42" s="99"/>
-      <c r="G42" s="99"/>
-      <c r="H42" s="99"/>
-      <c r="I42" s="99"/>
-      <c r="J42" s="100"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="32"/>
+      <c r="J42" s="33"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B43" s="101" t="s">
+      <c r="B43" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="101"/>
-      <c r="D43" s="101" t="s">
+      <c r="C43" s="34"/>
+      <c r="D43" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="E43" s="101"/>
-      <c r="F43" s="101"/>
-      <c r="G43" s="101"/>
-      <c r="H43" s="101"/>
-      <c r="I43" s="101" t="s">
+      <c r="E43" s="34"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="34"/>
+      <c r="H43" s="34"/>
+      <c r="I43" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J43" s="101"/>
+      <c r="J43" s="34"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B44" s="87"/>
-      <c r="C44" s="87"/>
-      <c r="D44" s="87"/>
-      <c r="E44" s="87"/>
-      <c r="F44" s="87"/>
-      <c r="G44" s="87"/>
-      <c r="H44" s="87"/>
-      <c r="I44" s="87"/>
-      <c r="J44" s="87"/>
+      <c r="B44" s="19"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="19"/>
+      <c r="G44" s="19"/>
+      <c r="H44" s="19"/>
+      <c r="I44" s="19"/>
+      <c r="J44" s="19"/>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B45" s="87"/>
-      <c r="C45" s="87"/>
-      <c r="D45" s="87"/>
-      <c r="E45" s="87"/>
-      <c r="F45" s="87"/>
-      <c r="G45" s="87"/>
-      <c r="H45" s="87"/>
-      <c r="I45" s="87"/>
-      <c r="J45" s="87"/>
+      <c r="B45" s="19"/>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
+      <c r="G45" s="19"/>
+      <c r="H45" s="19"/>
+      <c r="I45" s="19"/>
+      <c r="J45" s="19"/>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B46" s="87"/>
-      <c r="C46" s="87"/>
-      <c r="D46" s="87"/>
-      <c r="E46" s="87"/>
-      <c r="F46" s="87"/>
-      <c r="G46" s="87"/>
-      <c r="H46" s="87"/>
-      <c r="I46" s="87"/>
-      <c r="J46" s="87"/>
+      <c r="B46" s="19"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
+      <c r="G46" s="19"/>
+      <c r="H46" s="19"/>
+      <c r="I46" s="19"/>
+      <c r="J46" s="19"/>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B47" s="87"/>
-      <c r="C47" s="87"/>
-      <c r="D47" s="87"/>
-      <c r="E47" s="87"/>
-      <c r="F47" s="87"/>
-      <c r="G47" s="87"/>
-      <c r="H47" s="87"/>
-      <c r="I47" s="87"/>
-      <c r="J47" s="87"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
+      <c r="F47" s="19"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="19"/>
+      <c r="I47" s="19"/>
+      <c r="J47" s="19"/>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B48" s="87"/>
-      <c r="C48" s="87"/>
-      <c r="D48" s="87"/>
-      <c r="E48" s="87"/>
-      <c r="F48" s="87"/>
-      <c r="G48" s="87"/>
-      <c r="H48" s="87"/>
-      <c r="I48" s="87"/>
-      <c r="J48" s="87"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="19"/>
+      <c r="G48" s="19"/>
+      <c r="H48" s="19"/>
+      <c r="I48" s="19"/>
+      <c r="J48" s="19"/>
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B49" s="87"/>
-      <c r="C49" s="87"/>
-      <c r="D49" s="87"/>
-      <c r="E49" s="87"/>
-      <c r="F49" s="87"/>
-      <c r="G49" s="87"/>
-      <c r="H49" s="87"/>
-      <c r="I49" s="87"/>
-      <c r="J49" s="87"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+      <c r="I49" s="19"/>
+      <c r="J49" s="19"/>
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B50" s="87"/>
-      <c r="C50" s="87"/>
-      <c r="D50" s="87"/>
-      <c r="E50" s="87"/>
-      <c r="F50" s="87"/>
-      <c r="G50" s="87"/>
-      <c r="H50" s="87"/>
-      <c r="I50" s="87"/>
-      <c r="J50" s="87"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+      <c r="I50" s="19"/>
+      <c r="J50" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="D48:H48"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="D46:H46"/>
-    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="B8:J9"/>
+    <mergeCell ref="B2:C5"/>
+    <mergeCell ref="D2:H5"/>
+    <mergeCell ref="I2:J3"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:G16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:G27"/>
     <mergeCell ref="B44:C44"/>
     <mergeCell ref="D44:H44"/>
     <mergeCell ref="I44:J44"/>
@@ -3350,48 +3310,24 @@
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="D43:H43"/>
     <mergeCell ref="I43:J43"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:G16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:G17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:G13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:G15"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="B8:J9"/>
-    <mergeCell ref="B2:C5"/>
-    <mergeCell ref="D2:H5"/>
-    <mergeCell ref="I2:J3"/>
-    <mergeCell ref="B6:J6"/>
-    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="D46:H46"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="D48:H48"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="I50:J50"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -3419,39 +3355,39 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="103" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
-      <c r="G2" s="104"/>
-      <c r="H2" s="105"/>
-      <c r="I2" s="112" t="s">
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="94" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="113"/>
+      <c r="J2" s="95"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="106"/>
-      <c r="E3" s="107"/>
-      <c r="F3" s="107"/>
-      <c r="G3" s="107"/>
-      <c r="H3" s="108"/>
-      <c r="I3" s="114"/>
-      <c r="J3" s="115"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="96"/>
+      <c r="J3" s="97"/>
     </row>
     <row r="4" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="106"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="107"/>
-      <c r="H4" s="108"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="88"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="89"/>
+      <c r="G4" s="89"/>
+      <c r="H4" s="90"/>
       <c r="I4" s="10" t="s">
         <v>16</v>
       </c>
@@ -3460,13 +3396,13 @@
       </c>
     </row>
     <row r="5" spans="2:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="109"/>
-      <c r="E5" s="110"/>
-      <c r="F5" s="110"/>
-      <c r="G5" s="110"/>
-      <c r="H5" s="111"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="92"/>
+      <c r="F5" s="92"/>
+      <c r="G5" s="92"/>
+      <c r="H5" s="93"/>
       <c r="I5" s="9" t="s">
         <v>29</v>
       </c>
@@ -3475,53 +3411,53 @@
       </c>
     </row>
     <row r="6" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="98" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="39"/>
-      <c r="J6" s="39"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="98"/>
+      <c r="E6" s="98"/>
+      <c r="F6" s="98"/>
+      <c r="G6" s="98"/>
+      <c r="H6" s="98"/>
+      <c r="I6" s="98"/>
+      <c r="J6" s="98"/>
     </row>
     <row r="7" spans="2:10" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="116" t="s">
+      <c r="B7" s="99" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="39"/>
+      <c r="C7" s="98"/>
+      <c r="D7" s="98"/>
+      <c r="E7" s="98"/>
+      <c r="F7" s="98"/>
+      <c r="G7" s="98"/>
+      <c r="H7" s="98"/>
+      <c r="I7" s="98"/>
+      <c r="J7" s="98"/>
     </row>
     <row r="8" spans="2:10" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="39"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="39"/>
-      <c r="J8" s="39"/>
+      <c r="B8" s="98"/>
+      <c r="C8" s="98"/>
+      <c r="D8" s="98"/>
+      <c r="E8" s="98"/>
+      <c r="F8" s="98"/>
+      <c r="G8" s="98"/>
+      <c r="H8" s="98"/>
+      <c r="I8" s="98"/>
+      <c r="J8" s="98"/>
     </row>
     <row r="9" spans="2:10" s="8" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="102" t="s">
+      <c r="B9" s="84" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="102"/>
-      <c r="D9" s="102" t="s">
+      <c r="C9" s="84"/>
+      <c r="D9" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="102"/>
-      <c r="F9" s="102"/>
-      <c r="G9" s="102"/>
+      <c r="E9" s="84"/>
+      <c r="F9" s="84"/>
+      <c r="G9" s="84"/>
       <c r="H9" s="12" t="s">
         <v>1</v>
       </c>
@@ -3533,551 +3469,572 @@
       </c>
     </row>
     <row r="10" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="117"/>
-      <c r="C10" s="118"/>
-      <c r="D10" s="117"/>
-      <c r="E10" s="119"/>
-      <c r="F10" s="119"/>
-      <c r="G10" s="118"/>
+      <c r="B10" s="81"/>
+      <c r="C10" s="82"/>
+      <c r="D10" s="81"/>
+      <c r="E10" s="83"/>
+      <c r="F10" s="83"/>
+      <c r="G10" s="82"/>
       <c r="H10" s="4"/>
       <c r="I10" s="2"/>
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="117"/>
-      <c r="C11" s="118"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="119"/>
-      <c r="F11" s="119"/>
-      <c r="G11" s="118"/>
+      <c r="B11" s="81"/>
+      <c r="C11" s="82"/>
+      <c r="D11" s="81"/>
+      <c r="E11" s="83"/>
+      <c r="F11" s="83"/>
+      <c r="G11" s="82"/>
       <c r="H11" s="4"/>
       <c r="I11" s="2"/>
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="117"/>
-      <c r="C12" s="118"/>
-      <c r="D12" s="117"/>
-      <c r="E12" s="119"/>
-      <c r="F12" s="119"/>
-      <c r="G12" s="118"/>
+      <c r="B12" s="81"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="81"/>
+      <c r="E12" s="83"/>
+      <c r="F12" s="83"/>
+      <c r="G12" s="82"/>
       <c r="H12" s="4"/>
       <c r="I12" s="2"/>
       <c r="J12" s="3"/>
     </row>
     <row r="13" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="117"/>
-      <c r="C13" s="118"/>
-      <c r="D13" s="117"/>
-      <c r="E13" s="119"/>
-      <c r="F13" s="119"/>
-      <c r="G13" s="118"/>
+      <c r="B13" s="81"/>
+      <c r="C13" s="82"/>
+      <c r="D13" s="81"/>
+      <c r="E13" s="83"/>
+      <c r="F13" s="83"/>
+      <c r="G13" s="82"/>
       <c r="H13" s="4"/>
       <c r="I13" s="2"/>
       <c r="J13" s="3"/>
     </row>
     <row r="14" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="117"/>
-      <c r="C14" s="118"/>
-      <c r="D14" s="117"/>
-      <c r="E14" s="119"/>
-      <c r="F14" s="119"/>
-      <c r="G14" s="118"/>
+      <c r="B14" s="81"/>
+      <c r="C14" s="82"/>
+      <c r="D14" s="81"/>
+      <c r="E14" s="83"/>
+      <c r="F14" s="83"/>
+      <c r="G14" s="82"/>
       <c r="H14" s="4"/>
       <c r="I14" s="2"/>
       <c r="J14" s="3"/>
     </row>
     <row r="15" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="117"/>
-      <c r="C15" s="118"/>
-      <c r="D15" s="117"/>
-      <c r="E15" s="119"/>
-      <c r="F15" s="119"/>
-      <c r="G15" s="118"/>
+      <c r="B15" s="81"/>
+      <c r="C15" s="82"/>
+      <c r="D15" s="81"/>
+      <c r="E15" s="83"/>
+      <c r="F15" s="83"/>
+      <c r="G15" s="82"/>
       <c r="H15" s="4"/>
       <c r="I15" s="2"/>
       <c r="J15" s="3"/>
     </row>
     <row r="16" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="117"/>
-      <c r="C16" s="118"/>
-      <c r="D16" s="117"/>
-      <c r="E16" s="119"/>
-      <c r="F16" s="119"/>
-      <c r="G16" s="118"/>
+      <c r="B16" s="81"/>
+      <c r="C16" s="82"/>
+      <c r="D16" s="81"/>
+      <c r="E16" s="83"/>
+      <c r="F16" s="83"/>
+      <c r="G16" s="82"/>
       <c r="H16" s="4"/>
       <c r="I16" s="2"/>
       <c r="J16" s="3"/>
     </row>
     <row r="17" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
     </row>
     <row r="25" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
     </row>
     <row r="26" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
     </row>
     <row r="27" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="25"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="25"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
     </row>
     <row r="28" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
     </row>
     <row r="29" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="25"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
     </row>
     <row r="31" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="25"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B32" s="58" t="s">
+      <c r="B32" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="C32" s="58"/>
-      <c r="D32" s="58"/>
-      <c r="E32" s="58"/>
-      <c r="F32" s="58"/>
-      <c r="G32" s="58"/>
-      <c r="H32" s="58"/>
-      <c r="I32" s="58"/>
-      <c r="J32" s="58"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
+      <c r="G32" s="62"/>
+      <c r="H32" s="62"/>
+      <c r="I32" s="62"/>
+      <c r="J32" s="62"/>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B33" s="58"/>
-      <c r="C33" s="58"/>
-      <c r="D33" s="58"/>
-      <c r="E33" s="58"/>
-      <c r="F33" s="58"/>
-      <c r="G33" s="58"/>
-      <c r="H33" s="58"/>
-      <c r="I33" s="58"/>
-      <c r="J33" s="58"/>
+      <c r="B33" s="62"/>
+      <c r="C33" s="62"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="62"/>
+      <c r="G33" s="62"/>
+      <c r="H33" s="62"/>
+      <c r="I33" s="62"/>
+      <c r="J33" s="62"/>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B34" s="58"/>
-      <c r="C34" s="58"/>
-      <c r="D34" s="58"/>
-      <c r="E34" s="58"/>
-      <c r="F34" s="58"/>
-      <c r="G34" s="58"/>
-      <c r="H34" s="58"/>
-      <c r="I34" s="58"/>
-      <c r="J34" s="58"/>
+      <c r="B34" s="62"/>
+      <c r="C34" s="62"/>
+      <c r="D34" s="62"/>
+      <c r="E34" s="62"/>
+      <c r="F34" s="62"/>
+      <c r="G34" s="62"/>
+      <c r="H34" s="62"/>
+      <c r="I34" s="62"/>
+      <c r="J34" s="62"/>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B35" s="58"/>
-      <c r="C35" s="58"/>
-      <c r="D35" s="58"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="58"/>
-      <c r="G35" s="58"/>
-      <c r="H35" s="58"/>
-      <c r="I35" s="58"/>
-      <c r="J35" s="58"/>
+      <c r="B35" s="62"/>
+      <c r="C35" s="62"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="62"/>
+      <c r="F35" s="62"/>
+      <c r="G35" s="62"/>
+      <c r="H35" s="62"/>
+      <c r="I35" s="62"/>
+      <c r="J35" s="62"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="49" t="s">
+      <c r="B36" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="C36" s="50"/>
-      <c r="D36" s="50"/>
-      <c r="E36" s="50"/>
-      <c r="F36" s="50"/>
-      <c r="G36" s="50"/>
-      <c r="H36" s="50"/>
-      <c r="I36" s="50"/>
-      <c r="J36" s="51"/>
+      <c r="C36" s="64"/>
+      <c r="D36" s="64"/>
+      <c r="E36" s="64"/>
+      <c r="F36" s="64"/>
+      <c r="G36" s="64"/>
+      <c r="H36" s="64"/>
+      <c r="I36" s="64"/>
+      <c r="J36" s="65"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="52"/>
-      <c r="C37" s="53"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="53"/>
-      <c r="G37" s="53"/>
-      <c r="H37" s="53"/>
-      <c r="I37" s="53"/>
-      <c r="J37" s="54"/>
+      <c r="B37" s="66"/>
+      <c r="C37" s="67"/>
+      <c r="D37" s="67"/>
+      <c r="E37" s="67"/>
+      <c r="F37" s="67"/>
+      <c r="G37" s="67"/>
+      <c r="H37" s="67"/>
+      <c r="I37" s="67"/>
+      <c r="J37" s="68"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="52"/>
-      <c r="C38" s="53"/>
-      <c r="D38" s="53"/>
-      <c r="E38" s="53"/>
-      <c r="F38" s="53"/>
-      <c r="G38" s="53"/>
-      <c r="H38" s="53"/>
-      <c r="I38" s="53"/>
-      <c r="J38" s="54"/>
+      <c r="B38" s="66"/>
+      <c r="C38" s="67"/>
+      <c r="D38" s="67"/>
+      <c r="E38" s="67"/>
+      <c r="F38" s="67"/>
+      <c r="G38" s="67"/>
+      <c r="H38" s="67"/>
+      <c r="I38" s="67"/>
+      <c r="J38" s="68"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="55"/>
-      <c r="C39" s="56"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="56"/>
-      <c r="H39" s="56"/>
-      <c r="I39" s="56"/>
-      <c r="J39" s="57"/>
+      <c r="B39" s="69"/>
+      <c r="C39" s="70"/>
+      <c r="D39" s="70"/>
+      <c r="E39" s="70"/>
+      <c r="F39" s="70"/>
+      <c r="G39" s="70"/>
+      <c r="H39" s="70"/>
+      <c r="I39" s="70"/>
+      <c r="J39" s="71"/>
     </row>
     <row r="40" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="60" t="s">
+      <c r="B40" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="C40" s="61"/>
-      <c r="D40" s="61"/>
-      <c r="E40" s="61"/>
-      <c r="F40" s="61"/>
-      <c r="G40" s="61"/>
-      <c r="H40" s="61"/>
-      <c r="I40" s="61"/>
-      <c r="J40" s="62"/>
+      <c r="C40" s="73"/>
+      <c r="D40" s="73"/>
+      <c r="E40" s="73"/>
+      <c r="F40" s="73"/>
+      <c r="G40" s="73"/>
+      <c r="H40" s="73"/>
+      <c r="I40" s="73"/>
+      <c r="J40" s="74"/>
     </row>
     <row r="41" spans="2:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="63"/>
-      <c r="C41" s="64"/>
-      <c r="D41" s="64"/>
-      <c r="E41" s="64"/>
-      <c r="F41" s="64"/>
-      <c r="G41" s="64"/>
-      <c r="H41" s="64"/>
-      <c r="I41" s="64"/>
-      <c r="J41" s="65"/>
+      <c r="B41" s="75"/>
+      <c r="C41" s="76"/>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="76"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="76"/>
+      <c r="I41" s="76"/>
+      <c r="J41" s="77"/>
     </row>
     <row r="42" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="66"/>
-      <c r="C42" s="67"/>
-      <c r="D42" s="67"/>
-      <c r="E42" s="67"/>
-      <c r="F42" s="67"/>
-      <c r="G42" s="67"/>
-      <c r="H42" s="67"/>
-      <c r="I42" s="67"/>
-      <c r="J42" s="68"/>
+      <c r="B42" s="78"/>
+      <c r="C42" s="79"/>
+      <c r="D42" s="79"/>
+      <c r="E42" s="79"/>
+      <c r="F42" s="79"/>
+      <c r="G42" s="79"/>
+      <c r="H42" s="79"/>
+      <c r="I42" s="79"/>
+      <c r="J42" s="80"/>
     </row>
     <row r="43" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="59" t="s">
+      <c r="B43" s="61" t="s">
         <v>26</v>
       </c>
-      <c r="C43" s="58"/>
-      <c r="D43" s="58"/>
-      <c r="E43" s="58"/>
-      <c r="F43" s="58"/>
-      <c r="G43" s="58"/>
-      <c r="H43" s="58"/>
-      <c r="I43" s="58"/>
-      <c r="J43" s="58"/>
+      <c r="C43" s="62"/>
+      <c r="D43" s="62"/>
+      <c r="E43" s="62"/>
+      <c r="F43" s="62"/>
+      <c r="G43" s="62"/>
+      <c r="H43" s="62"/>
+      <c r="I43" s="62"/>
+      <c r="J43" s="62"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B44" s="58"/>
-      <c r="C44" s="58"/>
-      <c r="D44" s="58"/>
-      <c r="E44" s="58"/>
-      <c r="F44" s="58"/>
-      <c r="G44" s="58"/>
-      <c r="H44" s="58"/>
-      <c r="I44" s="58"/>
-      <c r="J44" s="58"/>
+      <c r="B44" s="62"/>
+      <c r="C44" s="62"/>
+      <c r="D44" s="62"/>
+      <c r="E44" s="62"/>
+      <c r="F44" s="62"/>
+      <c r="G44" s="62"/>
+      <c r="H44" s="62"/>
+      <c r="I44" s="62"/>
+      <c r="J44" s="62"/>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B45" s="58"/>
-      <c r="C45" s="58"/>
-      <c r="D45" s="58"/>
-      <c r="E45" s="58"/>
-      <c r="F45" s="58"/>
-      <c r="G45" s="58"/>
-      <c r="H45" s="58"/>
-      <c r="I45" s="58"/>
-      <c r="J45" s="58"/>
+      <c r="B45" s="62"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="62"/>
+      <c r="E45" s="62"/>
+      <c r="F45" s="62"/>
+      <c r="G45" s="62"/>
+      <c r="H45" s="62"/>
+      <c r="I45" s="62"/>
+      <c r="J45" s="62"/>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B46" s="58"/>
-      <c r="C46" s="58"/>
-      <c r="D46" s="58"/>
-      <c r="E46" s="58"/>
-      <c r="F46" s="58"/>
-      <c r="G46" s="58"/>
-      <c r="H46" s="58"/>
-      <c r="I46" s="58"/>
-      <c r="J46" s="58"/>
+      <c r="B46" s="62"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="62"/>
+      <c r="E46" s="62"/>
+      <c r="F46" s="62"/>
+      <c r="G46" s="62"/>
+      <c r="H46" s="62"/>
+      <c r="I46" s="62"/>
+      <c r="J46" s="62"/>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B47" s="58"/>
-      <c r="C47" s="58"/>
-      <c r="D47" s="58"/>
-      <c r="E47" s="58"/>
-      <c r="F47" s="58"/>
-      <c r="G47" s="58"/>
-      <c r="H47" s="58"/>
-      <c r="I47" s="58"/>
-      <c r="J47" s="58"/>
+      <c r="B47" s="62"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="62"/>
+      <c r="E47" s="62"/>
+      <c r="F47" s="62"/>
+      <c r="G47" s="62"/>
+      <c r="H47" s="62"/>
+      <c r="I47" s="62"/>
+      <c r="J47" s="62"/>
     </row>
     <row r="48" spans="2:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="120" t="s">
+      <c r="B48" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="C48" s="121"/>
-      <c r="D48" s="121"/>
-      <c r="E48" s="121"/>
-      <c r="F48" s="121"/>
-      <c r="G48" s="121"/>
-      <c r="H48" s="121"/>
-      <c r="I48" s="121"/>
-      <c r="J48" s="122"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="58"/>
+      <c r="G48" s="58"/>
+      <c r="H48" s="58"/>
+      <c r="I48" s="58"/>
+      <c r="J48" s="59"/>
     </row>
     <row r="49" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="123" t="s">
+      <c r="B49" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="C49" s="123"/>
-      <c r="D49" s="123" t="s">
+      <c r="C49" s="60"/>
+      <c r="D49" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="E49" s="123"/>
-      <c r="F49" s="123"/>
-      <c r="G49" s="123"/>
-      <c r="H49" s="123"/>
-      <c r="I49" s="123" t="s">
+      <c r="E49" s="60"/>
+      <c r="F49" s="60"/>
+      <c r="G49" s="60"/>
+      <c r="H49" s="60"/>
+      <c r="I49" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="J49" s="123"/>
+      <c r="J49" s="60"/>
     </row>
     <row r="50" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="124"/>
-      <c r="C50" s="124"/>
-      <c r="D50" s="124"/>
-      <c r="E50" s="124"/>
-      <c r="F50" s="124"/>
-      <c r="G50" s="124"/>
-      <c r="H50" s="124"/>
-      <c r="I50" s="124"/>
-      <c r="J50" s="124"/>
+      <c r="B50" s="53"/>
+      <c r="C50" s="53"/>
+      <c r="D50" s="53"/>
+      <c r="E50" s="53"/>
+      <c r="F50" s="53"/>
+      <c r="G50" s="53"/>
+      <c r="H50" s="53"/>
+      <c r="I50" s="53"/>
+      <c r="J50" s="53"/>
     </row>
     <row r="51" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="125"/>
-      <c r="C51" s="126"/>
-      <c r="D51" s="125"/>
-      <c r="E51" s="127"/>
-      <c r="F51" s="127"/>
-      <c r="G51" s="127"/>
-      <c r="H51" s="126"/>
-      <c r="I51" s="125"/>
-      <c r="J51" s="126"/>
+      <c r="B51" s="54"/>
+      <c r="C51" s="55"/>
+      <c r="D51" s="54"/>
+      <c r="E51" s="56"/>
+      <c r="F51" s="56"/>
+      <c r="G51" s="56"/>
+      <c r="H51" s="55"/>
+      <c r="I51" s="54"/>
+      <c r="J51" s="55"/>
     </row>
     <row r="52" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="124"/>
-      <c r="C52" s="124"/>
-      <c r="D52" s="124"/>
-      <c r="E52" s="124"/>
-      <c r="F52" s="124"/>
-      <c r="G52" s="124"/>
-      <c r="H52" s="124"/>
-      <c r="I52" s="124"/>
-      <c r="J52" s="124"/>
+      <c r="B52" s="53"/>
+      <c r="C52" s="53"/>
+      <c r="D52" s="53"/>
+      <c r="E52" s="53"/>
+      <c r="F52" s="53"/>
+      <c r="G52" s="53"/>
+      <c r="H52" s="53"/>
+      <c r="I52" s="53"/>
+      <c r="J52" s="53"/>
     </row>
     <row r="53" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="124"/>
-      <c r="C53" s="124"/>
-      <c r="D53" s="124"/>
-      <c r="E53" s="124"/>
-      <c r="F53" s="124"/>
-      <c r="G53" s="124"/>
-      <c r="H53" s="124"/>
-      <c r="I53" s="124"/>
-      <c r="J53" s="124"/>
+      <c r="B53" s="53"/>
+      <c r="C53" s="53"/>
+      <c r="D53" s="53"/>
+      <c r="E53" s="53"/>
+      <c r="F53" s="53"/>
+      <c r="G53" s="53"/>
+      <c r="H53" s="53"/>
+      <c r="I53" s="53"/>
+      <c r="J53" s="53"/>
     </row>
     <row r="54" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="124"/>
-      <c r="C54" s="124"/>
-      <c r="D54" s="124"/>
-      <c r="E54" s="124"/>
-      <c r="F54" s="124"/>
-      <c r="G54" s="124"/>
-      <c r="H54" s="124"/>
-      <c r="I54" s="124"/>
-      <c r="J54" s="124"/>
+      <c r="B54" s="53"/>
+      <c r="C54" s="53"/>
+      <c r="D54" s="53"/>
+      <c r="E54" s="53"/>
+      <c r="F54" s="53"/>
+      <c r="G54" s="53"/>
+      <c r="H54" s="53"/>
+      <c r="I54" s="53"/>
+      <c r="J54" s="53"/>
     </row>
     <row r="55" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="124"/>
-      <c r="C55" s="124"/>
-      <c r="D55" s="124"/>
-      <c r="E55" s="124"/>
-      <c r="F55" s="124"/>
-      <c r="G55" s="124"/>
-      <c r="H55" s="124"/>
-      <c r="I55" s="124"/>
-      <c r="J55" s="124"/>
+      <c r="B55" s="53"/>
+      <c r="C55" s="53"/>
+      <c r="D55" s="53"/>
+      <c r="E55" s="53"/>
+      <c r="F55" s="53"/>
+      <c r="G55" s="53"/>
+      <c r="H55" s="53"/>
+      <c r="I55" s="53"/>
+      <c r="J55" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="D55:H55"/>
-    <mergeCell ref="I55:J55"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="D53:H53"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="D54:H54"/>
-    <mergeCell ref="I54:J54"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="D51:H51"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="D52:H52"/>
-    <mergeCell ref="I52:J52"/>
-    <mergeCell ref="B48:J48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="D49:H49"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="D50:H50"/>
-    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="B2:C5"/>
+    <mergeCell ref="D2:H5"/>
+    <mergeCell ref="I2:J3"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="B7:J8"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:G16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:G27"/>
     <mergeCell ref="B43:J47"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="D28:G28"/>
@@ -4090,49 +4047,28 @@
     <mergeCell ref="B32:J35"/>
     <mergeCell ref="B36:J39"/>
     <mergeCell ref="B40:J42"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:G16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:G17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:G13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:G15"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="B2:C5"/>
-    <mergeCell ref="D2:H5"/>
-    <mergeCell ref="I2:J3"/>
-    <mergeCell ref="B6:J6"/>
-    <mergeCell ref="B7:J8"/>
+    <mergeCell ref="B48:J48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="D49:H49"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="D50:H50"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="D51:H51"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="D52:H52"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="D55:H55"/>
+    <mergeCell ref="I55:J55"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="D53:H53"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="D54:H54"/>
+    <mergeCell ref="I54:J54"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -4161,118 +4097,118 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="106" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="35" t="s">
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
+      <c r="H2" s="108"/>
+      <c r="I2" s="115" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="36"/>
-      <c r="K2" s="24"/>
+      <c r="J2" s="116"/>
+      <c r="K2" s="105"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="38"/>
-      <c r="K3" s="24"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="117"/>
+      <c r="J3" s="118"/>
+      <c r="K3" s="105"/>
     </row>
     <row r="4" spans="1:16" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="31"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="109"/>
+      <c r="E4" s="110"/>
+      <c r="F4" s="110"/>
+      <c r="G4" s="110"/>
+      <c r="H4" s="111"/>
       <c r="I4" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="24"/>
+      <c r="K4" s="105"/>
     </row>
     <row r="5" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="34"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="112"/>
+      <c r="E5" s="113"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="114"/>
       <c r="I5" s="9" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J5" s="13">
         <v>46245</v>
       </c>
-      <c r="K5" s="24"/>
+      <c r="K5" s="105"/>
     </row>
     <row r="6" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="39" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="39"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="24"/>
+      <c r="B6" s="98" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="98"/>
+      <c r="D6" s="98"/>
+      <c r="E6" s="98"/>
+      <c r="F6" s="98"/>
+      <c r="G6" s="98"/>
+      <c r="H6" s="98"/>
+      <c r="I6" s="98"/>
+      <c r="J6" s="98"/>
+      <c r="K6" s="105"/>
     </row>
     <row r="7" spans="1:16" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="119" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="46" t="s">
+      <c r="C7" s="120"/>
+      <c r="D7" s="120"/>
+      <c r="E7" s="120"/>
+      <c r="F7" s="120"/>
+      <c r="G7" s="120"/>
+      <c r="H7" s="120"/>
+      <c r="I7" s="121"/>
+      <c r="J7" s="125" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="24"/>
+      <c r="K7" s="105"/>
     </row>
     <row r="8" spans="1:16" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="43"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
-      <c r="I8" s="45"/>
-      <c r="J8" s="47"/>
-      <c r="K8" s="24"/>
+      <c r="B8" s="122"/>
+      <c r="C8" s="123"/>
+      <c r="D8" s="123"/>
+      <c r="E8" s="123"/>
+      <c r="F8" s="123"/>
+      <c r="G8" s="123"/>
+      <c r="H8" s="123"/>
+      <c r="I8" s="124"/>
+      <c r="J8" s="126"/>
+      <c r="K8" s="105"/>
     </row>
     <row r="9" spans="1:16" s="8" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="127" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="48"/>
-      <c r="D9" s="48" t="s">
+      <c r="C9" s="127"/>
+      <c r="D9" s="127" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48"/>
-      <c r="G9" s="48"/>
+      <c r="E9" s="127"/>
+      <c r="F9" s="127"/>
+      <c r="G9" s="127"/>
       <c r="H9" s="14" t="s">
         <v>1</v>
       </c>
@@ -4282,19 +4218,19 @@
       <c r="J9" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="K9" s="24"/>
+      <c r="K9" s="105"/>
     </row>
     <row r="10" spans="1:16" s="8" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="20"/>
-      <c r="D10" s="21" t="s">
+      <c r="B10" s="100" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="101"/>
+      <c r="D10" s="102" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="23"/>
+      <c r="E10" s="103"/>
+      <c r="F10" s="103"/>
+      <c r="G10" s="104"/>
       <c r="H10" s="16">
         <v>4</v>
       </c>
@@ -4304,751 +4240,698 @@
       <c r="J10" s="17">
         <v>5</v>
       </c>
-      <c r="K10" s="24"/>
+      <c r="K10" s="105"/>
     </row>
     <row r="11" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="16">
-        <v>4</v>
-      </c>
-      <c r="I11" s="16">
-        <v>2</v>
-      </c>
-      <c r="J11" s="17">
-        <v>5</v>
-      </c>
-      <c r="K11" s="24"/>
+      <c r="B11" s="100"/>
+      <c r="C11" s="101"/>
+      <c r="D11" s="102"/>
+      <c r="E11" s="103"/>
+      <c r="F11" s="103"/>
+      <c r="G11" s="104"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="105"/>
       <c r="P11" s="18"/>
     </row>
     <row r="12" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
-      <c r="B12" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="20"/>
-      <c r="D12" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="16">
-        <v>4</v>
-      </c>
-      <c r="I12" s="16">
-        <v>2</v>
-      </c>
-      <c r="J12" s="17">
-        <v>5</v>
-      </c>
-      <c r="K12" s="24"/>
+      <c r="B12" s="100"/>
+      <c r="C12" s="101"/>
+      <c r="D12" s="102"/>
+      <c r="E12" s="103"/>
+      <c r="F12" s="103"/>
+      <c r="G12" s="104"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="105"/>
     </row>
     <row r="13" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="16">
-        <v>4</v>
-      </c>
-      <c r="I13" s="16">
-        <v>2</v>
-      </c>
-      <c r="J13" s="17">
-        <v>5</v>
-      </c>
-      <c r="K13" s="24"/>
+      <c r="B13" s="100"/>
+      <c r="C13" s="101"/>
+      <c r="D13" s="102"/>
+      <c r="E13" s="103"/>
+      <c r="F13" s="103"/>
+      <c r="G13" s="104"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="105"/>
     </row>
     <row r="14" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
-      <c r="B14" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="16">
-        <v>4</v>
-      </c>
-      <c r="I14" s="16">
-        <v>2</v>
-      </c>
-      <c r="J14" s="17">
-        <v>5</v>
-      </c>
-      <c r="K14" s="24"/>
+      <c r="B14" s="100"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="102"/>
+      <c r="E14" s="103"/>
+      <c r="F14" s="103"/>
+      <c r="G14" s="104"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="105"/>
     </row>
     <row r="15" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="16">
-        <v>4</v>
-      </c>
-      <c r="I15" s="16">
-        <v>2</v>
-      </c>
-      <c r="J15" s="17">
-        <v>5</v>
-      </c>
-      <c r="K15" s="24"/>
+      <c r="B15" s="100"/>
+      <c r="C15" s="101"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
+      <c r="F15" s="103"/>
+      <c r="G15" s="104"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="105"/>
     </row>
     <row r="16" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
-      <c r="B16" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="16">
-        <v>4</v>
-      </c>
-      <c r="I16" s="16">
-        <v>2</v>
-      </c>
-      <c r="J16" s="17">
-        <v>5</v>
-      </c>
-      <c r="K16" s="24"/>
+      <c r="B16" s="100"/>
+      <c r="C16" s="101"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
+      <c r="F16" s="103"/>
+      <c r="G16" s="104"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="105"/>
     </row>
     <row r="17" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="16">
-        <v>4</v>
-      </c>
-      <c r="I17" s="16">
-        <v>2</v>
-      </c>
-      <c r="J17" s="17">
-        <v>5</v>
-      </c>
-      <c r="K17" s="24"/>
+      <c r="B17" s="100"/>
+      <c r="C17" s="101"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
+      <c r="F17" s="103"/>
+      <c r="G17" s="104"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="105"/>
     </row>
     <row r="18" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
-      <c r="B18" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="20"/>
-      <c r="D18" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="16">
-        <v>4</v>
-      </c>
-      <c r="I18" s="16">
-        <v>2</v>
-      </c>
-      <c r="J18" s="17">
-        <v>5</v>
-      </c>
-      <c r="K18" s="24"/>
+      <c r="B18" s="100"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
+      <c r="F18" s="103"/>
+      <c r="G18" s="104"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="105"/>
     </row>
     <row r="19" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="16">
-        <v>4</v>
-      </c>
-      <c r="I19" s="16">
-        <v>2</v>
-      </c>
-      <c r="J19" s="17">
-        <v>5</v>
-      </c>
-      <c r="K19" s="24"/>
+      <c r="B19" s="100"/>
+      <c r="C19" s="101"/>
+      <c r="D19" s="102"/>
+      <c r="E19" s="103"/>
+      <c r="F19" s="103"/>
+      <c r="G19" s="104"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="105"/>
     </row>
     <row r="20" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
-      <c r="B20" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="16">
-        <v>4</v>
-      </c>
-      <c r="I20" s="16">
-        <v>2</v>
-      </c>
-      <c r="J20" s="17">
-        <v>5</v>
-      </c>
-      <c r="K20" s="24"/>
+      <c r="B20" s="100"/>
+      <c r="C20" s="101"/>
+      <c r="D20" s="102"/>
+      <c r="E20" s="103"/>
+      <c r="F20" s="103"/>
+      <c r="G20" s="104"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="105"/>
     </row>
     <row r="21" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="16">
-        <v>4</v>
-      </c>
-      <c r="I21" s="16">
-        <v>2</v>
-      </c>
-      <c r="J21" s="17">
-        <v>5</v>
-      </c>
-      <c r="K21" s="24"/>
+      <c r="B21" s="100"/>
+      <c r="C21" s="101"/>
+      <c r="D21" s="102"/>
+      <c r="E21" s="103"/>
+      <c r="F21" s="103"/>
+      <c r="G21" s="104"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="105"/>
     </row>
     <row r="22" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8"/>
-      <c r="B22" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="20"/>
-      <c r="D22" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="16">
-        <v>4</v>
-      </c>
-      <c r="I22" s="16">
-        <v>2</v>
-      </c>
-      <c r="J22" s="17">
-        <v>5</v>
-      </c>
-      <c r="K22" s="24"/>
+      <c r="B22" s="100"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="102"/>
+      <c r="E22" s="103"/>
+      <c r="F22" s="103"/>
+      <c r="G22" s="104"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="105"/>
     </row>
     <row r="23" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="19"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="23"/>
+      <c r="B23" s="100"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="102"/>
+      <c r="E23" s="103"/>
+      <c r="F23" s="103"/>
+      <c r="G23" s="104"/>
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
       <c r="J23" s="17"/>
-      <c r="K23" s="24"/>
+      <c r="K23" s="105"/>
     </row>
     <row r="24" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="23"/>
+      <c r="B24" s="100"/>
+      <c r="C24" s="101"/>
+      <c r="D24" s="102"/>
+      <c r="E24" s="103"/>
+      <c r="F24" s="103"/>
+      <c r="G24" s="104"/>
       <c r="H24" s="16"/>
       <c r="I24" s="16"/>
       <c r="J24" s="17"/>
-      <c r="K24" s="24"/>
+      <c r="K24" s="105"/>
     </row>
     <row r="25" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="19"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="23"/>
+      <c r="B25" s="100"/>
+      <c r="C25" s="101"/>
+      <c r="D25" s="102"/>
+      <c r="E25" s="103"/>
+      <c r="F25" s="103"/>
+      <c r="G25" s="104"/>
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="17"/>
-      <c r="K25" s="24"/>
+      <c r="K25" s="105"/>
     </row>
     <row r="26" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="23"/>
+      <c r="B26" s="100"/>
+      <c r="C26" s="101"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="103"/>
+      <c r="F26" s="103"/>
+      <c r="G26" s="104"/>
       <c r="H26" s="16"/>
       <c r="I26" s="16"/>
       <c r="J26" s="17"/>
-      <c r="K26" s="24"/>
+      <c r="K26" s="105"/>
     </row>
     <row r="27" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="19"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="23"/>
+      <c r="B27" s="100"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="102"/>
+      <c r="E27" s="103"/>
+      <c r="F27" s="103"/>
+      <c r="G27" s="104"/>
       <c r="H27" s="16"/>
       <c r="I27" s="16"/>
       <c r="J27" s="17"/>
-      <c r="K27" s="24"/>
+      <c r="K27" s="105"/>
     </row>
     <row r="28" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="23"/>
+      <c r="B28" s="100"/>
+      <c r="C28" s="101"/>
+      <c r="D28" s="102"/>
+      <c r="E28" s="103"/>
+      <c r="F28" s="103"/>
+      <c r="G28" s="104"/>
       <c r="H28" s="16"/>
       <c r="I28" s="16"/>
       <c r="J28" s="17"/>
-      <c r="K28" s="24"/>
+      <c r="K28" s="105"/>
     </row>
     <row r="29" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="19"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="23"/>
+      <c r="B29" s="100"/>
+      <c r="C29" s="101"/>
+      <c r="D29" s="102"/>
+      <c r="E29" s="103"/>
+      <c r="F29" s="103"/>
+      <c r="G29" s="104"/>
       <c r="H29" s="16"/>
       <c r="I29" s="16"/>
       <c r="J29" s="17"/>
-      <c r="K29" s="24"/>
+      <c r="K29" s="105"/>
     </row>
     <row r="30" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="23"/>
+      <c r="B30" s="100"/>
+      <c r="C30" s="101"/>
+      <c r="D30" s="102"/>
+      <c r="E30" s="103"/>
+      <c r="F30" s="103"/>
+      <c r="G30" s="104"/>
       <c r="H30" s="16"/>
       <c r="I30" s="16"/>
       <c r="J30" s="17"/>
-      <c r="K30" s="24"/>
+      <c r="K30" s="105"/>
     </row>
     <row r="31" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="19"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
-      <c r="G31" s="23"/>
+      <c r="B31" s="100"/>
+      <c r="C31" s="101"/>
+      <c r="D31" s="102"/>
+      <c r="E31" s="103"/>
+      <c r="F31" s="103"/>
+      <c r="G31" s="104"/>
       <c r="H31" s="16"/>
       <c r="I31" s="16"/>
       <c r="J31" s="17"/>
-      <c r="K31" s="24"/>
+      <c r="K31" s="105"/>
     </row>
     <row r="32" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="23"/>
+      <c r="B32" s="100"/>
+      <c r="C32" s="101"/>
+      <c r="D32" s="102"/>
+      <c r="E32" s="103"/>
+      <c r="F32" s="103"/>
+      <c r="G32" s="104"/>
       <c r="H32" s="16"/>
       <c r="I32" s="16"/>
       <c r="J32" s="17"/>
-      <c r="K32" s="24"/>
+      <c r="K32" s="105"/>
     </row>
     <row r="33" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="19"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="23"/>
+      <c r="B33" s="100"/>
+      <c r="C33" s="101"/>
+      <c r="D33" s="102"/>
+      <c r="E33" s="103"/>
+      <c r="F33" s="103"/>
+      <c r="G33" s="104"/>
       <c r="H33" s="16"/>
       <c r="I33" s="16"/>
       <c r="J33" s="17"/>
-      <c r="K33" s="24"/>
+      <c r="K33" s="105"/>
     </row>
     <row r="34" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="19"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="23"/>
+      <c r="B34" s="100"/>
+      <c r="C34" s="101"/>
+      <c r="D34" s="102"/>
+      <c r="E34" s="103"/>
+      <c r="F34" s="103"/>
+      <c r="G34" s="104"/>
       <c r="H34" s="16"/>
       <c r="I34" s="16"/>
       <c r="J34" s="17"/>
-      <c r="K34" s="24"/>
+      <c r="K34" s="105"/>
     </row>
     <row r="35" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="19"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="23"/>
+      <c r="B35" s="100"/>
+      <c r="C35" s="101"/>
+      <c r="D35" s="102"/>
+      <c r="E35" s="103"/>
+      <c r="F35" s="103"/>
+      <c r="G35" s="104"/>
       <c r="H35" s="16"/>
       <c r="I35" s="16"/>
       <c r="J35" s="17"/>
-      <c r="K35" s="24"/>
+      <c r="K35" s="105"/>
     </row>
     <row r="36" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="19"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="23"/>
+      <c r="B36" s="100"/>
+      <c r="C36" s="101"/>
+      <c r="D36" s="102"/>
+      <c r="E36" s="103"/>
+      <c r="F36" s="103"/>
+      <c r="G36" s="104"/>
       <c r="H36" s="16"/>
       <c r="I36" s="16"/>
       <c r="J36" s="17"/>
-      <c r="K36" s="24"/>
+      <c r="K36" s="105"/>
     </row>
     <row r="37" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="19"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="23"/>
+      <c r="B37" s="100"/>
+      <c r="C37" s="101"/>
+      <c r="D37" s="102"/>
+      <c r="E37" s="103"/>
+      <c r="F37" s="103"/>
+      <c r="G37" s="104"/>
       <c r="H37" s="16"/>
       <c r="I37" s="16"/>
       <c r="J37" s="17"/>
-      <c r="K37" s="24"/>
+      <c r="K37" s="105"/>
     </row>
     <row r="38" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="19"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="23"/>
+      <c r="B38" s="100"/>
+      <c r="C38" s="101"/>
+      <c r="D38" s="102"/>
+      <c r="E38" s="103"/>
+      <c r="F38" s="103"/>
+      <c r="G38" s="104"/>
       <c r="H38" s="16"/>
       <c r="I38" s="16"/>
       <c r="J38" s="17"/>
-      <c r="K38" s="24"/>
+      <c r="K38" s="105"/>
     </row>
     <row r="39" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="19"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="23"/>
+      <c r="B39" s="100"/>
+      <c r="C39" s="101"/>
+      <c r="D39" s="102"/>
+      <c r="E39" s="103"/>
+      <c r="F39" s="103"/>
+      <c r="G39" s="104"/>
       <c r="H39" s="16"/>
       <c r="I39" s="16"/>
       <c r="J39" s="17"/>
-      <c r="K39" s="24"/>
+      <c r="K39" s="105"/>
     </row>
     <row r="40" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="19"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="23"/>
+      <c r="B40" s="100"/>
+      <c r="C40" s="101"/>
+      <c r="D40" s="102"/>
+      <c r="E40" s="103"/>
+      <c r="F40" s="103"/>
+      <c r="G40" s="104"/>
       <c r="H40" s="16"/>
       <c r="I40" s="16"/>
       <c r="J40" s="17"/>
-      <c r="K40" s="24"/>
+      <c r="K40" s="105"/>
     </row>
     <row r="41" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="19"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="23"/>
+      <c r="B41" s="100"/>
+      <c r="C41" s="101"/>
+      <c r="D41" s="102"/>
+      <c r="E41" s="103"/>
+      <c r="F41" s="103"/>
+      <c r="G41" s="104"/>
       <c r="H41" s="16"/>
       <c r="I41" s="16"/>
       <c r="J41" s="17"/>
-      <c r="K41" s="24"/>
+      <c r="K41" s="105"/>
     </row>
     <row r="42" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="19"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="21"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="23"/>
+      <c r="B42" s="100"/>
+      <c r="C42" s="101"/>
+      <c r="D42" s="102"/>
+      <c r="E42" s="103"/>
+      <c r="F42" s="103"/>
+      <c r="G42" s="104"/>
       <c r="H42" s="16"/>
       <c r="I42" s="16"/>
       <c r="J42" s="17"/>
-      <c r="K42" s="24"/>
+      <c r="K42" s="105"/>
     </row>
     <row r="43" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="19"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="21"/>
-      <c r="E43" s="22"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="23"/>
+      <c r="B43" s="100"/>
+      <c r="C43" s="101"/>
+      <c r="D43" s="102"/>
+      <c r="E43" s="103"/>
+      <c r="F43" s="103"/>
+      <c r="G43" s="104"/>
       <c r="H43" s="16"/>
       <c r="I43" s="16"/>
       <c r="J43" s="17"/>
-      <c r="K43" s="24"/>
+      <c r="K43" s="105"/>
     </row>
     <row r="44" spans="2:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="19"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="23"/>
+      <c r="B44" s="100"/>
+      <c r="C44" s="101"/>
+      <c r="D44" s="102"/>
+      <c r="E44" s="103"/>
+      <c r="F44" s="103"/>
+      <c r="G44" s="104"/>
       <c r="H44" s="16"/>
       <c r="I44" s="16"/>
       <c r="J44" s="17"/>
-      <c r="K44" s="24"/>
+      <c r="K44" s="105"/>
     </row>
     <row r="45" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B45" s="58" t="s">
+      <c r="B45" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="C45" s="58"/>
-      <c r="D45" s="58"/>
-      <c r="E45" s="58"/>
-      <c r="F45" s="58"/>
-      <c r="G45" s="58"/>
-      <c r="H45" s="58"/>
-      <c r="I45" s="58"/>
-      <c r="J45" s="58"/>
-      <c r="K45" s="24"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="62"/>
+      <c r="E45" s="62"/>
+      <c r="F45" s="62"/>
+      <c r="G45" s="62"/>
+      <c r="H45" s="62"/>
+      <c r="I45" s="62"/>
+      <c r="J45" s="62"/>
+      <c r="K45" s="105"/>
     </row>
     <row r="46" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B46" s="58"/>
-      <c r="C46" s="58"/>
-      <c r="D46" s="58"/>
-      <c r="E46" s="58"/>
-      <c r="F46" s="58"/>
-      <c r="G46" s="58"/>
-      <c r="H46" s="58"/>
-      <c r="I46" s="58"/>
-      <c r="J46" s="58"/>
-      <c r="K46" s="24"/>
+      <c r="B46" s="62"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="62"/>
+      <c r="E46" s="62"/>
+      <c r="F46" s="62"/>
+      <c r="G46" s="62"/>
+      <c r="H46" s="62"/>
+      <c r="I46" s="62"/>
+      <c r="J46" s="62"/>
+      <c r="K46" s="105"/>
     </row>
     <row r="47" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B47" s="58"/>
-      <c r="C47" s="58"/>
-      <c r="D47" s="58"/>
-      <c r="E47" s="58"/>
-      <c r="F47" s="58"/>
-      <c r="G47" s="58"/>
-      <c r="H47" s="58"/>
-      <c r="I47" s="58"/>
-      <c r="J47" s="58"/>
-      <c r="K47" s="24"/>
+      <c r="B47" s="62"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="62"/>
+      <c r="E47" s="62"/>
+      <c r="F47" s="62"/>
+      <c r="G47" s="62"/>
+      <c r="H47" s="62"/>
+      <c r="I47" s="62"/>
+      <c r="J47" s="62"/>
+      <c r="K47" s="105"/>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B48" s="58"/>
-      <c r="C48" s="58"/>
-      <c r="D48" s="58"/>
-      <c r="E48" s="58"/>
-      <c r="F48" s="58"/>
-      <c r="G48" s="58"/>
-      <c r="H48" s="58"/>
-      <c r="I48" s="58"/>
-      <c r="J48" s="58"/>
-      <c r="K48" s="24"/>
+      <c r="B48" s="62"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="62"/>
+      <c r="G48" s="62"/>
+      <c r="H48" s="62"/>
+      <c r="I48" s="62"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="105"/>
     </row>
     <row r="49" spans="2:11" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="49" t="s">
+      <c r="B49" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="C49" s="50"/>
-      <c r="D49" s="50"/>
-      <c r="E49" s="50"/>
-      <c r="F49" s="50"/>
-      <c r="G49" s="50"/>
-      <c r="H49" s="50"/>
-      <c r="I49" s="50"/>
-      <c r="J49" s="51"/>
-      <c r="K49" s="24"/>
+      <c r="C49" s="64"/>
+      <c r="D49" s="64"/>
+      <c r="E49" s="64"/>
+      <c r="F49" s="64"/>
+      <c r="G49" s="64"/>
+      <c r="H49" s="64"/>
+      <c r="I49" s="64"/>
+      <c r="J49" s="65"/>
+      <c r="K49" s="105"/>
     </row>
     <row r="50" spans="2:11" ht="41.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="52"/>
-      <c r="C50" s="53"/>
-      <c r="D50" s="53"/>
-      <c r="E50" s="53"/>
-      <c r="F50" s="53"/>
-      <c r="G50" s="53"/>
-      <c r="H50" s="53"/>
-      <c r="I50" s="53"/>
-      <c r="J50" s="54"/>
-      <c r="K50" s="24"/>
+      <c r="B50" s="66"/>
+      <c r="C50" s="67"/>
+      <c r="D50" s="67"/>
+      <c r="E50" s="67"/>
+      <c r="F50" s="67"/>
+      <c r="G50" s="67"/>
+      <c r="H50" s="67"/>
+      <c r="I50" s="67"/>
+      <c r="J50" s="68"/>
+      <c r="K50" s="105"/>
     </row>
     <row r="51" spans="2:11" ht="0.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="52"/>
-      <c r="C51" s="53"/>
-      <c r="D51" s="53"/>
-      <c r="E51" s="53"/>
-      <c r="F51" s="53"/>
-      <c r="G51" s="53"/>
-      <c r="H51" s="53"/>
-      <c r="I51" s="53"/>
-      <c r="J51" s="54"/>
-      <c r="K51" s="24"/>
+      <c r="B51" s="66"/>
+      <c r="C51" s="67"/>
+      <c r="D51" s="67"/>
+      <c r="E51" s="67"/>
+      <c r="F51" s="67"/>
+      <c r="G51" s="67"/>
+      <c r="H51" s="67"/>
+      <c r="I51" s="67"/>
+      <c r="J51" s="68"/>
+      <c r="K51" s="105"/>
     </row>
     <row r="52" spans="2:11" ht="41.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="55"/>
-      <c r="C52" s="56"/>
-      <c r="D52" s="56"/>
-      <c r="E52" s="56"/>
-      <c r="F52" s="56"/>
-      <c r="G52" s="56"/>
-      <c r="H52" s="56"/>
-      <c r="I52" s="56"/>
-      <c r="J52" s="57"/>
-      <c r="K52" s="24"/>
+      <c r="B52" s="69"/>
+      <c r="C52" s="70"/>
+      <c r="D52" s="70"/>
+      <c r="E52" s="70"/>
+      <c r="F52" s="70"/>
+      <c r="G52" s="70"/>
+      <c r="H52" s="70"/>
+      <c r="I52" s="70"/>
+      <c r="J52" s="71"/>
+      <c r="K52" s="105"/>
     </row>
     <row r="53" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="60" t="s">
+      <c r="B53" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="C53" s="61"/>
-      <c r="D53" s="61"/>
-      <c r="E53" s="61"/>
-      <c r="F53" s="61"/>
-      <c r="G53" s="61"/>
-      <c r="H53" s="61"/>
-      <c r="I53" s="61"/>
-      <c r="J53" s="62"/>
-      <c r="K53" s="24"/>
+      <c r="C53" s="73"/>
+      <c r="D53" s="73"/>
+      <c r="E53" s="73"/>
+      <c r="F53" s="73"/>
+      <c r="G53" s="73"/>
+      <c r="H53" s="73"/>
+      <c r="I53" s="73"/>
+      <c r="J53" s="74"/>
+      <c r="K53" s="105"/>
     </row>
     <row r="54" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="63"/>
-      <c r="C54" s="64"/>
-      <c r="D54" s="64"/>
-      <c r="E54" s="64"/>
-      <c r="F54" s="64"/>
-      <c r="G54" s="64"/>
-      <c r="H54" s="64"/>
-      <c r="I54" s="64"/>
-      <c r="J54" s="65"/>
-      <c r="K54" s="24"/>
+      <c r="B54" s="75"/>
+      <c r="C54" s="76"/>
+      <c r="D54" s="76"/>
+      <c r="E54" s="76"/>
+      <c r="F54" s="76"/>
+      <c r="G54" s="76"/>
+      <c r="H54" s="76"/>
+      <c r="I54" s="76"/>
+      <c r="J54" s="77"/>
+      <c r="K54" s="105"/>
     </row>
     <row r="55" spans="2:11" ht="5.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="66"/>
-      <c r="C55" s="67"/>
-      <c r="D55" s="67"/>
-      <c r="E55" s="67"/>
-      <c r="F55" s="67"/>
-      <c r="G55" s="67"/>
-      <c r="H55" s="67"/>
-      <c r="I55" s="67"/>
-      <c r="J55" s="68"/>
-      <c r="K55" s="24"/>
+      <c r="B55" s="78"/>
+      <c r="C55" s="79"/>
+      <c r="D55" s="79"/>
+      <c r="E55" s="79"/>
+      <c r="F55" s="79"/>
+      <c r="G55" s="79"/>
+      <c r="H55" s="79"/>
+      <c r="I55" s="79"/>
+      <c r="J55" s="80"/>
+      <c r="K55" s="105"/>
     </row>
     <row r="56" spans="2:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="59" t="s">
+      <c r="B56" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="C56" s="58"/>
-      <c r="D56" s="58"/>
-      <c r="E56" s="58"/>
-      <c r="F56" s="58"/>
-      <c r="G56" s="58"/>
-      <c r="H56" s="58"/>
-      <c r="I56" s="58"/>
-      <c r="J56" s="58"/>
-      <c r="K56" s="24"/>
+      <c r="C56" s="62"/>
+      <c r="D56" s="62"/>
+      <c r="E56" s="62"/>
+      <c r="F56" s="62"/>
+      <c r="G56" s="62"/>
+      <c r="H56" s="62"/>
+      <c r="I56" s="62"/>
+      <c r="J56" s="62"/>
+      <c r="K56" s="105"/>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B57" s="58"/>
-      <c r="C57" s="58"/>
-      <c r="D57" s="58"/>
-      <c r="E57" s="58"/>
-      <c r="F57" s="58"/>
-      <c r="G57" s="58"/>
-      <c r="H57" s="58"/>
-      <c r="I57" s="58"/>
-      <c r="J57" s="58"/>
-      <c r="K57" s="24"/>
+      <c r="B57" s="62"/>
+      <c r="C57" s="62"/>
+      <c r="D57" s="62"/>
+      <c r="E57" s="62"/>
+      <c r="F57" s="62"/>
+      <c r="G57" s="62"/>
+      <c r="H57" s="62"/>
+      <c r="I57" s="62"/>
+      <c r="J57" s="62"/>
+      <c r="K57" s="105"/>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B58" s="58"/>
-      <c r="C58" s="58"/>
-      <c r="D58" s="58"/>
-      <c r="E58" s="58"/>
-      <c r="F58" s="58"/>
-      <c r="G58" s="58"/>
-      <c r="H58" s="58"/>
-      <c r="I58" s="58"/>
-      <c r="J58" s="58"/>
-      <c r="K58" s="24"/>
+      <c r="B58" s="62"/>
+      <c r="C58" s="62"/>
+      <c r="D58" s="62"/>
+      <c r="E58" s="62"/>
+      <c r="F58" s="62"/>
+      <c r="G58" s="62"/>
+      <c r="H58" s="62"/>
+      <c r="I58" s="62"/>
+      <c r="J58" s="62"/>
+      <c r="K58" s="105"/>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B59" s="58"/>
-      <c r="C59" s="58"/>
-      <c r="D59" s="58"/>
-      <c r="E59" s="58"/>
-      <c r="F59" s="58"/>
-      <c r="G59" s="58"/>
-      <c r="H59" s="58"/>
-      <c r="I59" s="58"/>
-      <c r="J59" s="58"/>
-      <c r="K59" s="24"/>
+      <c r="B59" s="62"/>
+      <c r="C59" s="62"/>
+      <c r="D59" s="62"/>
+      <c r="E59" s="62"/>
+      <c r="F59" s="62"/>
+      <c r="G59" s="62"/>
+      <c r="H59" s="62"/>
+      <c r="I59" s="62"/>
+      <c r="J59" s="62"/>
+      <c r="K59" s="105"/>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B60" s="58"/>
-      <c r="C60" s="58"/>
-      <c r="D60" s="58"/>
-      <c r="E60" s="58"/>
-      <c r="F60" s="58"/>
-      <c r="G60" s="58"/>
-      <c r="H60" s="58"/>
-      <c r="I60" s="58"/>
-      <c r="J60" s="58"/>
-      <c r="K60" s="24"/>
+      <c r="B60" s="62"/>
+      <c r="C60" s="62"/>
+      <c r="D60" s="62"/>
+      <c r="E60" s="62"/>
+      <c r="F60" s="62"/>
+      <c r="G60" s="62"/>
+      <c r="H60" s="62"/>
+      <c r="I60" s="62"/>
+      <c r="J60" s="62"/>
+      <c r="K60" s="105"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="83">
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="K2:K60"/>
+    <mergeCell ref="B2:C5"/>
+    <mergeCell ref="D2:H5"/>
+    <mergeCell ref="I2:J3"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="B7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:G16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="B49:J52"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B45:J48"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:G28"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D30:G30"/>
+    <mergeCell ref="D31:G31"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="D43:G43"/>
+    <mergeCell ref="D35:G35"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D32:G32"/>
+    <mergeCell ref="D33:G33"/>
+    <mergeCell ref="D34:G34"/>
     <mergeCell ref="B44:C44"/>
     <mergeCell ref="D44:G44"/>
     <mergeCell ref="B56:J60"/>
@@ -5065,73 +4948,6 @@
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="D41:G41"/>
     <mergeCell ref="D42:G42"/>
-    <mergeCell ref="D43:G43"/>
-    <mergeCell ref="D35:G35"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D32:G32"/>
-    <mergeCell ref="D33:G33"/>
-    <mergeCell ref="D34:G34"/>
-    <mergeCell ref="B49:J52"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B45:J48"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:G28"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D30:G30"/>
-    <mergeCell ref="D31:G31"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="D16:G16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:G17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="K2:K60"/>
-    <mergeCell ref="B2:C5"/>
-    <mergeCell ref="D2:H5"/>
-    <mergeCell ref="I2:J3"/>
-    <mergeCell ref="B6:J6"/>
-    <mergeCell ref="B7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="D13:G13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:G15"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:G12"/>
   </mergeCells>
   <phoneticPr fontId="19" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>